<commit_message>
Allow for increased LCFS
-Include aviation
-Max LCFS in webapp is 50%, with updated text and caution
-Max blend is set to 100% for diesel, and increases to 100% by 2040 for planes, ships, & trains.
</commit_message>
<xml_diff>
--- a/InputData/trans/BVTStL/Boolean Veh Types Subject to LCFS.xlsx
+++ b/InputData/trans/BVTStL/Boolean Veh Types Subject to LCFS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10411"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10711"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/users/nathaniyer/library/containers/com.microsoft.excel/data/state-eps-data-repository/template_state/trans/bvtstl/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zsubin/Documents/Code/eps-newmexico/InputData/trans/BVTStL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F5A2312-0E57-BB4A-A964-3FB4326B4915}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A54300-E35B-484B-B832-4CA1AD0E9A0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="460" windowWidth="23960" windowHeight="11320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7960" yWindow="500" windowWidth="23960" windowHeight="11320" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -601,10 +601,10 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>